<commit_message>
update with more stuff
</commit_message>
<xml_diff>
--- a/LAB/data/Participant_information.xlsx
+++ b/LAB/data/Participant_information.xlsx
@@ -8,24 +8,38 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Martin\Documents\R\WebEye\LAB\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CBA6AA2-8D02-4CC9-863D-66C03B1BC7E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8706936F-A32C-4592-B176-29C1CE6AA448}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$H$51</definedName>
+  </definedNames>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="23">
   <si>
     <t>ID</t>
   </si>
@@ -88,9 +102,6 @@
   </si>
   <si>
     <t>D</t>
-  </si>
-  <si>
-    <t>replace</t>
   </si>
   <si>
     <t>replaced- bad calibration accuracy</t>
@@ -146,7 +157,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -168,12 +179,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -455,7 +460,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H51"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:H61"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="3" width="8.7265625" style="1"/>
@@ -488,10 +494,10 @@
         <v>4</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" s="7">
         <v>1</v>
       </c>
@@ -526,6 +532,9 @@
       <c r="G3" s="1" t="s">
         <v>9</v>
       </c>
+      <c r="H3" s="1" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
@@ -549,6 +558,9 @@
       <c r="G4" s="1" t="s">
         <v>9</v>
       </c>
+      <c r="H4" s="1" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
@@ -572,30 +584,33 @@
       <c r="G5" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A6" s="8">
-        <v>5</v>
-      </c>
-      <c r="B6" s="8" t="s">
+      <c r="H5" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="1">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="8">
+      <c r="C6" s="1">
         <v>25</v>
       </c>
-      <c r="D6" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="E6" s="9">
+      <c r="D6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" s="4">
         <v>45545</v>
       </c>
-      <c r="F6" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="G6" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="H6" s="8" t="s">
+      <c r="F6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H6" s="1" t="s">
         <v>6</v>
       </c>
     </row>
@@ -617,6 +632,9 @@
       </c>
       <c r="F7" s="1" t="s">
         <v>6</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
@@ -638,6 +656,9 @@
       <c r="F8" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="H8" s="1" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="1">
@@ -658,8 +679,11 @@
       <c r="F9" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H9" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -682,10 +706,10 @@
         <v>13</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -704,8 +728,8 @@
       <c r="F11" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="G11" s="8" t="s">
-        <v>22</v>
+      <c r="G11" s="1" t="s">
+        <v>21</v>
       </c>
       <c r="H11" s="1" t="s">
         <v>6</v>
@@ -730,8 +754,11 @@
       <c r="F12" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H12" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -752,6 +779,9 @@
       </c>
       <c r="G13" s="1" t="s">
         <v>15</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
@@ -773,6 +803,9 @@
       <c r="F14" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="H14" s="1" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" s="1">
@@ -793,8 +826,11 @@
       <c r="F15" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H15" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" s="1">
         <v>15</v>
       </c>
@@ -802,8 +838,11 @@
       <c r="G16" s="1" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H16" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" s="1">
         <v>16</v>
       </c>
@@ -811,6 +850,9 @@
       <c r="G17" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="H17" s="1" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" s="1">
@@ -834,6 +876,9 @@
       <c r="G18" s="1" t="s">
         <v>16</v>
       </c>
+      <c r="H18" s="1" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" s="1">
@@ -854,6 +899,9 @@
       <c r="F19" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="H19" s="1" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" s="1">
@@ -873,6 +921,9 @@
       </c>
       <c r="F20" s="1" t="s">
         <v>6</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.35">
@@ -894,6 +945,9 @@
       <c r="F21" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="H21" s="1" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" s="1">
@@ -914,6 +968,9 @@
       <c r="F22" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="H22" s="1" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" s="1">
@@ -934,6 +991,9 @@
       <c r="F23" s="1" t="s">
         <v>12</v>
       </c>
+      <c r="H23" s="1" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" s="1">
@@ -954,8 +1014,11 @@
       <c r="F24" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H24" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" s="1">
         <v>24</v>
       </c>
@@ -975,7 +1038,7 @@
         <v>12</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H25" s="1" t="s">
         <v>6</v>
@@ -1000,6 +1063,9 @@
       <c r="F26" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="H26" s="1" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" s="1">
@@ -1020,6 +1086,9 @@
       <c r="F27" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="H27" s="1" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28" s="1">
@@ -1040,6 +1109,9 @@
       <c r="F28" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="H28" s="1" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" s="1">
@@ -1060,6 +1132,9 @@
       <c r="F29" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="H29" s="1" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30" s="1">
@@ -1080,6 +1155,9 @@
       <c r="F30" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="H30" s="1" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31" s="1">
@@ -1100,6 +1178,9 @@
       <c r="F31" s="1" t="s">
         <v>12</v>
       </c>
+      <c r="H31" s="1" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32" s="1">
@@ -1120,8 +1201,11 @@
       <c r="F32" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="H32" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A33" s="1">
         <v>32</v>
       </c>
@@ -1140,8 +1224,11 @@
       <c r="F33" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="H33" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A34" s="1">
         <v>33</v>
       </c>
@@ -1160,8 +1247,11 @@
       <c r="F34" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="H34" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A35" s="1">
         <v>34</v>
       </c>
@@ -1180,8 +1270,11 @@
       <c r="F35" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="H35" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A36" s="1">
         <v>35</v>
       </c>
@@ -1200,8 +1293,11 @@
       <c r="F36" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="H36" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A37" s="1">
         <v>36</v>
       </c>
@@ -1220,8 +1316,11 @@
       <c r="F37" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="H37" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A38" s="1">
         <v>37</v>
       </c>
@@ -1240,8 +1339,11 @@
       <c r="F38" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="H38" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A39" s="1">
         <v>38</v>
       </c>
@@ -1260,8 +1362,11 @@
       <c r="F39" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="H39" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A40" s="1">
         <v>39</v>
       </c>
@@ -1280,8 +1385,11 @@
       <c r="F40" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="H40" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A41" s="1">
         <v>40</v>
       </c>
@@ -1300,8 +1408,11 @@
       <c r="F41" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="H41" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A42" s="1">
         <v>41</v>
       </c>
@@ -1320,8 +1431,11 @@
       <c r="F42" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="H42" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A43" s="1">
         <v>42</v>
       </c>
@@ -1340,8 +1454,11 @@
       <c r="F43" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="H43" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A44" s="1">
         <v>43</v>
       </c>
@@ -1360,8 +1477,11 @@
       <c r="F44" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="H44" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A45" s="1">
         <v>44</v>
       </c>
@@ -1380,8 +1500,11 @@
       <c r="F45" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="H45" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A46" s="1">
         <v>45</v>
       </c>
@@ -1400,8 +1523,11 @@
       <c r="F46" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="H46" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A47" s="1">
         <v>46</v>
       </c>
@@ -1420,8 +1546,11 @@
       <c r="F47" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="H47" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A48" s="1">
         <v>47</v>
       </c>
@@ -1440,8 +1569,11 @@
       <c r="F48" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="H48" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A49" s="1">
         <v>48</v>
       </c>
@@ -1460,8 +1592,11 @@
       <c r="F49" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="H49" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A50" s="1">
         <v>49</v>
       </c>
@@ -1480,8 +1615,11 @@
       <c r="F50" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="H50" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A51" s="1">
         <v>50</v>
       </c>
@@ -1500,8 +1638,42 @@
       <c r="F51" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="H51" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="C56" s="1">
+        <f>AVERAGE(C18:C55)</f>
+        <v>24.735294117647058</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="C57" s="1">
+        <f>STDEV(C3:C51)</f>
+        <v>7.5772351655219996</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="C58" s="1">
+        <f>MIN(C3:C52)</f>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="C61" s="1">
+        <f>MAX(C4:C51)</f>
+        <v>49</v>
+      </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:H51" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="7">
+      <filters>
+        <filter val="Yes"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>